<commit_message>
file tmp KHNV, màn hình duyệt
</commit_message>
<xml_diff>
--- a/web/EXCEL_TEMPLATE/KHNV/KHNV_DK02.xlsx
+++ b/web/EXCEL_TEMPLATE/KHNV/KHNV_DK02.xlsx
@@ -5,7 +5,7 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Source_tree\IMS_REPORTS\build\web\EXCEL_TEMPLATE\KHNV\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ADMIN\Desktop\Cap nhat\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -68,7 +68,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="256" uniqueCount="218">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="258" uniqueCount="221">
   <si>
     <t>CỘNG HOÀ XÃ HỘI CHỦ NGHĨA VIỆT NAM</t>
   </si>
@@ -818,6 +818,15 @@
   </si>
   <si>
     <t>Biểu số 02A/NHCS-KH</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cho vay hộ gia đình SXKD tại VKK theo QĐ 31/2007/QĐ-TTg </t>
+  </si>
+  <si>
+    <t>XD000291</t>
+  </si>
+  <si>
+    <t>XD000251</t>
   </si>
 </sst>
 </file>
@@ -3046,7 +3055,7 @@
       <c r="E24" s="88"/>
       <c r="F24" s="88"/>
       <c r="G24" s="58">
-        <f t="shared" ref="G24:G50" si="2">F24-E24</f>
+        <f t="shared" ref="G24:G51" si="2">F24-E24</f>
         <v>0</v>
       </c>
       <c r="H24" s="55">
@@ -3978,15 +3987,23 @@
     </row>
     <row r="47" spans="1:52" ht="22.5" customHeight="1">
       <c r="A47" s="17"/>
-      <c r="B47" s="17"/>
+      <c r="B47" s="17" t="s">
+        <v>220</v>
+      </c>
       <c r="C47" s="98" t="s">
         <v>98</v>
       </c>
       <c r="D47" s="88"/>
       <c r="E47" s="88"/>
       <c r="F47" s="88"/>
-      <c r="G47" s="58"/>
-      <c r="H47" s="55"/>
+      <c r="G47" s="58">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="H47" s="55">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
     </row>
     <row r="48" spans="1:52" s="11" customFormat="1" ht="32.25" customHeight="1">
       <c r="A48" s="17">
@@ -4190,15 +4207,23 @@
       <c r="A51" s="17">
         <v>25</v>
       </c>
-      <c r="B51" s="17"/>
+      <c r="B51" s="17" t="s">
+        <v>219</v>
+      </c>
       <c r="C51" s="102" t="s">
         <v>92</v>
       </c>
       <c r="D51" s="88"/>
       <c r="E51" s="88"/>
       <c r="F51" s="88"/>
-      <c r="G51" s="58"/>
-      <c r="H51" s="55"/>
+      <c r="G51" s="58">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="H51" s="55">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
       <c r="I51" s="2"/>
       <c r="J51" s="2"/>
       <c r="K51" s="2"/>
@@ -4971,7 +4996,7 @@
         <v>171</v>
       </c>
       <c r="C78" s="68" t="s">
-        <v>62</v>
+        <v>218</v>
       </c>
       <c r="D78" s="88"/>
       <c r="E78" s="88"/>

</xml_diff>